<commit_message>
add files accreditamento and data.json
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDIBRIDGEXX/InnovaTeraSolutions/MEDIBRIDGE/1.0/accreditamento-checklist_V9.0.0.xlsx
+++ b/GATEWAY/A1#111#MEDIBRIDGEXX/InnovaTeraSolutions/MEDIBRIDGE/1.0/accreditamento-checklist_V9.0.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Startup\DigitalTwin\Accreditamento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E02A1A6-2615-49D9-B584-CA6929245ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55F935B-1493-438F-9058-D2E1940BEDEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -932,40 +932,40 @@
     <t>Timeout di rete</t>
   </si>
   <si>
-    <t>51743781e305fd40a81ba42616183c96</t>
-  </si>
-  <si>
-    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.03cfbe368a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>01/04/2026T21:52:23</t>
-  </si>
-  <si>
-    <t>01/04/2026T21:54:36</t>
-  </si>
-  <si>
-    <t>474689bfbfe1d3dab38e2d54d7e62bac</t>
-  </si>
-  <si>
-    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.77c6462407^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>66a8c067f3a04f41a36db2dc07eca5bc</t>
-  </si>
-  <si>
-    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.44c69e7cac^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>01/04/2026T22:10:41</t>
-  </si>
-  <si>
-    <t>98cf12c20bb20c08e2b3be1fe4f52cff</t>
-  </si>
-  <si>
-    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.a763856686^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>01/04/2026T22:11:46</t>
+    <t>e027ad2b34f348b416818b7f313a0157</t>
+  </si>
+  <si>
+    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.9cec6e8551^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>09/04/2026T20:03:43</t>
+  </si>
+  <si>
+    <t>5d4e4e7a6529bf11fc41f43c5de4eb09</t>
+  </si>
+  <si>
+    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.caf76ef2f7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>09/04/2026T20:07:04</t>
+  </si>
+  <si>
+    <t>68d949e35ad34f7b9051d92e1417bee5</t>
+  </si>
+  <si>
+    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.1de80fb597^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>09/04/2026T20:11:12</t>
+  </si>
+  <si>
+    <t>7e2bd8e6ae3d45859504176f19f338f3</t>
+  </si>
+  <si>
+    <t>IT-REG-LOM-01.1f2714c26a31f53a7de0221ad47cd5d24a96ebf759286393a89723d2697fe25e.a56fa87d14^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>09/04/2026T20:14:17</t>
   </si>
 </sst>
 </file>
@@ -975,7 +975,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1090,6 +1090,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1634,8 +1641,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5034,12 +5041,12 @@
         <v>125</v>
       </c>
       <c r="F47" s="28">
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="G47" s="28" t="s">
         <v>220</v>
       </c>
-      <c r="H47" s="61" t="s">
+      <c r="H47" s="48" t="s">
         <v>218</v>
       </c>
       <c r="I47" s="48" t="s">
@@ -5081,16 +5088,16 @@
         <v>127</v>
       </c>
       <c r="F48" s="28">
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="G48" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="H48" s="48" t="s">
         <v>221</v>
       </c>
-      <c r="H48" s="48" t="s">
+      <c r="I48" s="48" t="s">
         <v>222</v>
-      </c>
-      <c r="I48" s="48" t="s">
-        <v>223</v>
       </c>
       <c r="J48" s="29" t="s">
         <v>60</v>
@@ -5250,7 +5257,7 @@
         <v>135</v>
       </c>
       <c r="F52" s="28">
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="G52" s="28" t="s">
         <v>226</v>
@@ -5297,7 +5304,7 @@
         <v>137</v>
       </c>
       <c r="F53" s="28">
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="G53" s="28" t="s">
         <v>229</v>
@@ -5451,7 +5458,7 @@
     </row>
     <row r="58" spans="1:23" ht="14.25" customHeight="1">
       <c r="F58" s="6"/>
-      <c r="G58" s="6"/>
+      <c r="G58" s="61"/>
       <c r="H58" s="6"/>
       <c r="I58" s="6"/>
       <c r="J58" s="7"/>
@@ -9938,12 +9945,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10211,21 +10221,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10250,18 +10266,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>